<commit_message>
Test: kleiner Test für Reproduzierbarkeit des Scrapings basierend auf Offline-Caches
</commit_message>
<xml_diff>
--- a/src/evaluation/data/Backup/gpt_advanced/run_1/ragas_results_20260128_122607.xlsx
+++ b/src/evaluation/data/Backup/gpt_advanced/run_1/ragas_results_20260128_122607.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Uni-Köln\Masterarbeit\Software\uzk-masterarbeit\src\evaluation\data\Backup\gpt_advanced\run_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DD64927-C0B2-4045-8516-F34EAF75A903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F32C5D1-0AF8-46E3-9663-C3493D76E405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Detaillierte Ergebnisse" sheetId="1" r:id="rId1"/>
@@ -2471,7 +2471,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:AA117"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2577,7 +2576,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2660,7 +2659,7 @@
         <v>23.63501596450806</v>
       </c>
     </row>
-    <row r="3" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2743,7 +2742,7 @@
         <v>14.965632200241091</v>
       </c>
     </row>
-    <row r="4" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2826,7 +2825,7 @@
         <v>15.43052291870117</v>
       </c>
     </row>
-    <row r="5" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2909,7 +2908,7 @@
         <v>13.808202266693121</v>
       </c>
     </row>
-    <row r="6" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2992,7 +2991,7 @@
         <v>12.533143520355219</v>
       </c>
     </row>
-    <row r="7" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -3075,7 +3074,7 @@
         <v>19.096912622451779</v>
       </c>
     </row>
-    <row r="8" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -3158,7 +3157,7 @@
         <v>12.209736824035639</v>
       </c>
     </row>
-    <row r="9" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -3241,7 +3240,7 @@
         <v>15.10346388816833</v>
       </c>
     </row>
-    <row r="10" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -3324,7 +3323,7 @@
         <v>12.20202159881592</v>
       </c>
     </row>
-    <row r="11" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -3490,7 +3489,7 @@
         <v>13.946332216262819</v>
       </c>
     </row>
-    <row r="13" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -3573,7 +3572,7 @@
         <v>9.6785056591033936</v>
       </c>
     </row>
-    <row r="14" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -3656,7 +3655,7 @@
         <v>11.38377857208252</v>
       </c>
     </row>
-    <row r="15" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -3739,7 +3738,7 @@
         <v>10.95947051048279</v>
       </c>
     </row>
-    <row r="16" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3822,7 +3821,7 @@
         <v>19.703711748123169</v>
       </c>
     </row>
-    <row r="17" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -3905,7 +3904,7 @@
         <v>13.803689479827881</v>
       </c>
     </row>
-    <row r="18" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -3988,7 +3987,7 @@
         <v>10.828209161758419</v>
       </c>
     </row>
-    <row r="19" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -4071,7 +4070,7 @@
         <v>9.8454351425170898</v>
       </c>
     </row>
-    <row r="20" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -4154,7 +4153,7 @@
         <v>9.5628912448883057</v>
       </c>
     </row>
-    <row r="21" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -4237,7 +4236,7 @@
         <v>12.33128643035889</v>
       </c>
     </row>
-    <row r="22" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -4320,7 +4319,7 @@
         <v>15.05608916282654</v>
       </c>
     </row>
-    <row r="23" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -4403,7 +4402,7 @@
         <v>11.23437333106995</v>
       </c>
     </row>
-    <row r="24" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -4486,7 +4485,7 @@
         <v>12.353239774703979</v>
       </c>
     </row>
-    <row r="25" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -4569,7 +4568,7 @@
         <v>10.3865282535553</v>
       </c>
     </row>
-    <row r="26" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -4652,7 +4651,7 @@
         <v>14.58087420463562</v>
       </c>
     </row>
-    <row r="27" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -4735,7 +4734,7 @@
         <v>17.729062795639042</v>
       </c>
     </row>
-    <row r="28" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -4818,7 +4817,7 @@
         <v>10.39626669883728</v>
       </c>
     </row>
-    <row r="29" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -4901,7 +4900,7 @@
         <v>15.755085706710821</v>
       </c>
     </row>
-    <row r="30" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -4984,7 +4983,7 @@
         <v>14.573308706283569</v>
       </c>
     </row>
-    <row r="31" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -5067,7 +5066,7 @@
         <v>11.091047763824459</v>
       </c>
     </row>
-    <row r="32" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -5150,7 +5149,7 @@
         <v>12.50648045539856</v>
       </c>
     </row>
-    <row r="33" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -5233,7 +5232,7 @@
         <v>12.0364716053009</v>
       </c>
     </row>
-    <row r="34" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -5316,7 +5315,7 @@
         <v>8.5543985366821289</v>
       </c>
     </row>
-    <row r="35" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -5399,7 +5398,7 @@
         <v>14.24388575553894</v>
       </c>
     </row>
-    <row r="36" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -5482,7 +5481,7 @@
         <v>14.270649909973139</v>
       </c>
     </row>
-    <row r="37" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -5565,7 +5564,7 @@
         <v>12.645973443984991</v>
       </c>
     </row>
-    <row r="38" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -5648,7 +5647,7 @@
         <v>14.70406913757324</v>
       </c>
     </row>
-    <row r="39" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -5814,7 +5813,7 @@
         <v>13.364343404769899</v>
       </c>
     </row>
-    <row r="41" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -5897,7 +5896,7 @@
         <v>11.54607486724854</v>
       </c>
     </row>
-    <row r="42" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -5980,7 +5979,7 @@
         <v>9.3441917896270752</v>
       </c>
     </row>
-    <row r="43" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -6063,7 +6062,7 @@
         <v>13.179346561431879</v>
       </c>
     </row>
-    <row r="44" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -6146,7 +6145,7 @@
         <v>7.5131306648254386</v>
       </c>
     </row>
-    <row r="45" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -6229,7 +6228,7 @@
         <v>18.716945171356201</v>
       </c>
     </row>
-    <row r="46" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -6312,7 +6311,7 @@
         <v>12.707013845443729</v>
       </c>
     </row>
-    <row r="47" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -6395,7 +6394,7 @@
         <v>12.280468702316281</v>
       </c>
     </row>
-    <row r="48" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -6478,7 +6477,7 @@
         <v>12.074725389480591</v>
       </c>
     </row>
-    <row r="49" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -6561,7 +6560,7 @@
         <v>20.494038343429569</v>
       </c>
     </row>
-    <row r="50" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -6644,7 +6643,7 @@
         <v>17.729601383209229</v>
       </c>
     </row>
-    <row r="51" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -6727,7 +6726,7 @@
         <v>12.601881980896</v>
       </c>
     </row>
-    <row r="52" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -6810,7 +6809,7 @@
         <v>21.4474983215332</v>
       </c>
     </row>
-    <row r="53" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
@@ -6893,7 +6892,7 @@
         <v>11.571918725967411</v>
       </c>
     </row>
-    <row r="54" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
@@ -6976,7 +6975,7 @@
         <v>12.165248394012449</v>
       </c>
     </row>
-    <row r="55" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
@@ -7059,7 +7058,7 @@
         <v>12.266968488693241</v>
       </c>
     </row>
-    <row r="56" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -7142,7 +7141,7 @@
         <v>8.0316476821899414</v>
       </c>
     </row>
-    <row r="57" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
@@ -7225,7 +7224,7 @@
         <v>8.5864987373352051</v>
       </c>
     </row>
-    <row r="58" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -7308,7 +7307,7 @@
         <v>13.557025194168091</v>
       </c>
     </row>
-    <row r="59" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
@@ -7391,7 +7390,7 @@
         <v>14.958858251571661</v>
       </c>
     </row>
-    <row r="60" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
@@ -7474,7 +7473,7 @@
         <v>13.14629602432251</v>
       </c>
     </row>
-    <row r="61" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
@@ -7557,7 +7556,7 @@
         <v>9.4231266975402832</v>
       </c>
     </row>
-    <row r="62" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
@@ -7640,7 +7639,7 @@
         <v>10.2422993183136</v>
       </c>
     </row>
-    <row r="63" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
@@ -7723,7 +7722,7 @@
         <v>10.99390769004822</v>
       </c>
     </row>
-    <row r="64" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
@@ -7806,7 +7805,7 @@
         <v>10.336126089096069</v>
       </c>
     </row>
-    <row r="65" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
@@ -7889,7 +7888,7 @@
         <v>10.68692421913147</v>
       </c>
     </row>
-    <row r="66" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
@@ -7972,7 +7971,7 @@
         <v>14.76854634284973</v>
       </c>
     </row>
-    <row r="67" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
@@ -8055,7 +8054,7 @@
         <v>8.3219501972198486</v>
       </c>
     </row>
-    <row r="68" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
@@ -8138,7 +8137,7 @@
         <v>15.20471858978271</v>
       </c>
     </row>
-    <row r="69" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
@@ -8221,7 +8220,7 @@
         <v>11.41972684860229</v>
       </c>
     </row>
-    <row r="70" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
@@ -8304,7 +8303,7 @@
         <v>13.030813694000241</v>
       </c>
     </row>
-    <row r="71" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
@@ -8387,7 +8386,7 @@
         <v>14.125198364257811</v>
       </c>
     </row>
-    <row r="72" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
@@ -8470,7 +8469,7 @@
         <v>19.49803256988525</v>
       </c>
     </row>
-    <row r="73" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
@@ -8553,7 +8552,7 @@
         <v>10.36129999160767</v>
       </c>
     </row>
-    <row r="74" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
@@ -8636,7 +8635,7 @@
         <v>11.030380964279169</v>
       </c>
     </row>
-    <row r="75" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
@@ -8719,7 +8718,7 @@
         <v>16.29729700088501</v>
       </c>
     </row>
-    <row r="76" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>75</v>
       </c>
@@ -8802,7 +8801,7 @@
         <v>11.66205906867981</v>
       </c>
     </row>
-    <row r="77" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>76</v>
       </c>
@@ -8885,7 +8884,7 @@
         <v>14.267824172973629</v>
       </c>
     </row>
-    <row r="78" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>77</v>
       </c>
@@ -8968,7 +8967,7 @@
         <v>13.82828855514526</v>
       </c>
     </row>
-    <row r="79" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>78</v>
       </c>
@@ -9051,7 +9050,7 @@
         <v>13.789353609085079</v>
       </c>
     </row>
-    <row r="80" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>79</v>
       </c>
@@ -9134,7 +9133,7 @@
         <v>9.0278053283691406</v>
       </c>
     </row>
-    <row r="81" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>80</v>
       </c>
@@ -9217,7 +9216,7 @@
         <v>13.200951337814329</v>
       </c>
     </row>
-    <row r="82" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>81</v>
       </c>
@@ -9300,7 +9299,7 @@
         <v>13.712689638137819</v>
       </c>
     </row>
-    <row r="83" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>82</v>
       </c>
@@ -9383,7 +9382,7 @@
         <v>18.343915939331051</v>
       </c>
     </row>
-    <row r="84" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>83</v>
       </c>
@@ -9466,7 +9465,7 @@
         <v>13.26220345497131</v>
       </c>
     </row>
-    <row r="85" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>84</v>
       </c>
@@ -9549,7 +9548,7 @@
         <v>14.402899026870729</v>
       </c>
     </row>
-    <row r="86" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>85</v>
       </c>
@@ -9632,7 +9631,7 @@
         <v>11.9968044757843</v>
       </c>
     </row>
-    <row r="87" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>86</v>
       </c>
@@ -9715,7 +9714,7 @@
         <v>22.206417798995972</v>
       </c>
     </row>
-    <row r="88" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>87</v>
       </c>
@@ -9798,7 +9797,7 @@
         <v>10.696088790893549</v>
       </c>
     </row>
-    <row r="89" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>88</v>
       </c>
@@ -9881,7 +9880,7 @@
         <v>13.73142886161804</v>
       </c>
     </row>
-    <row r="90" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>89</v>
       </c>
@@ -9964,7 +9963,7 @@
         <v>10.8777961730957</v>
       </c>
     </row>
-    <row r="91" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>90</v>
       </c>
@@ -10047,7 +10046,7 @@
         <v>16.01394701004028</v>
       </c>
     </row>
-    <row r="92" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>91</v>
       </c>
@@ -10130,7 +10129,7 @@
         <v>27.619379997253422</v>
       </c>
     </row>
-    <row r="93" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>92</v>
       </c>
@@ -10213,7 +10212,7 @@
         <v>17.85649943351746</v>
       </c>
     </row>
-    <row r="94" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>93</v>
       </c>
@@ -10296,7 +10295,7 @@
         <v>11.888934373855591</v>
       </c>
     </row>
-    <row r="95" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>94</v>
       </c>
@@ -10379,7 +10378,7 @@
         <v>11.66355872154236</v>
       </c>
     </row>
-    <row r="96" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>95</v>
       </c>
@@ -10462,7 +10461,7 @@
         <v>12.52585077285767</v>
       </c>
     </row>
-    <row r="97" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>96</v>
       </c>
@@ -10545,7 +10544,7 @@
         <v>14.364378452301031</v>
       </c>
     </row>
-    <row r="98" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>97</v>
       </c>
@@ -10628,7 +10627,7 @@
         <v>14.898599624633791</v>
       </c>
     </row>
-    <row r="99" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>98</v>
       </c>
@@ -10711,7 +10710,7 @@
         <v>15.40545701980591</v>
       </c>
     </row>
-    <row r="100" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>99</v>
       </c>
@@ -10794,7 +10793,7 @@
         <v>14.34566688537598</v>
       </c>
     </row>
-    <row r="101" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>100</v>
       </c>
@@ -10877,7 +10876,7 @@
         <v>15.47704148292542</v>
       </c>
     </row>
-    <row r="102" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>101</v>
       </c>
@@ -10960,7 +10959,7 @@
         <v>12.06157255172729</v>
       </c>
     </row>
-    <row r="103" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>102</v>
       </c>
@@ -11043,7 +11042,7 @@
         <v>11.990336656570429</v>
       </c>
     </row>
-    <row r="104" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>103</v>
       </c>
@@ -11126,7 +11125,7 @@
         <v>8.5666294097900391</v>
       </c>
     </row>
-    <row r="105" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>104</v>
       </c>
@@ -11209,7 +11208,7 @@
         <v>10.862676382064819</v>
       </c>
     </row>
-    <row r="106" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>105</v>
       </c>
@@ -11292,7 +11291,7 @@
         <v>13.23422026634216</v>
       </c>
     </row>
-    <row r="107" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>106</v>
       </c>
@@ -11375,7 +11374,7 @@
         <v>14.46770000457764</v>
       </c>
     </row>
-    <row r="108" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>107</v>
       </c>
@@ -11458,7 +11457,7 @@
         <v>12.38386869430542</v>
       </c>
     </row>
-    <row r="109" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>108</v>
       </c>
@@ -11541,7 +11540,7 @@
         <v>17.877335071563721</v>
       </c>
     </row>
-    <row r="110" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>109</v>
       </c>
@@ -11624,7 +11623,7 @@
         <v>15.0128448009491</v>
       </c>
     </row>
-    <row r="111" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>110</v>
       </c>
@@ -11707,7 +11706,7 @@
         <v>21.120368003845211</v>
       </c>
     </row>
-    <row r="112" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>111</v>
       </c>
@@ -11790,7 +11789,7 @@
         <v>9.1482808589935303</v>
       </c>
     </row>
-    <row r="113" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>112</v>
       </c>
@@ -11873,7 +11872,7 @@
         <v>9.1488862037658691</v>
       </c>
     </row>
-    <row r="114" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>113</v>
       </c>
@@ -11956,7 +11955,7 @@
         <v>13.62296295166016</v>
       </c>
     </row>
-    <row r="115" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>114</v>
       </c>
@@ -12039,7 +12038,7 @@
         <v>10.99480509757996</v>
       </c>
     </row>
-    <row r="116" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>115</v>
       </c>
@@ -12122,7 +12121,7 @@
         <v>15.2870762348175</v>
       </c>
     </row>
-    <row r="117" spans="1:27" ht="409.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:27" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>116</v>
       </c>
@@ -12206,14 +12205,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA117" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="11"/>
-        <filter val="39"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>